<commit_message>
filled: developers, deadlines, prices, addresses for 29 KMV projects + Гармония data
Data sourced from ZenSerp API queries, project websites (novostroi-kmv.ru,
gid.house, kvartal-pechorin.ru, ssgkuban.ru, xn----dtbkbkbhc6ailz5k.xn--p1ai,
tretyrim.ru, effect-development.ru, klenovaya-kmv.ru, aksioma-sz.ru) and
наш.дом.рф EISZHS listings.

Key fills:
- Застройщики: 27/29 KMV rows filled (excl. ул.Кл.Цеткин, Titul)
- Срок сдачи: 15/29 rows now have dates
- Этажность/корпуса: added for крупные проекты
- Адреса: added for most
- Гармония (row 8): area 32.7m², price from 3 038 400, застройщик СК Третий Рим
- Cols 32-41 (УТП/преимущества/риски/ипотека/рассрочка/доходность): filled all
</commit_message>
<xml_diff>
--- a/Baza_Nedvizhimost.xlsx
+++ b/Baza_Nedvizhimost.xlsx
@@ -1096,6 +1096,21 @@
       <c r="R9" s="1">
         <v>9</v>
       </c>
+      <c r="U9" s="1" t="str">
+        <v>32,7</v>
+      </c>
+      <c r="W9" s="1" t="str">
+        <v>1к/2к/3к</v>
+      </c>
+      <c r="X9" s="1" t="str">
+        <v>3 038 400</v>
+      </c>
+      <c r="Y9" s="1" t="str">
+        <v>5 900 000</v>
+      </c>
+      <c r="AC9" s="1" t="str">
+        <v>3 038 400</v>
+      </c>
       <c r="AD9" s="1" t="str">
         <v>апрель 2026</v>
       </c>
@@ -1103,7 +1118,7 @@
         <v>Без отделки</v>
       </c>
       <c r="AF9" s="1" t="str">
-        <v>0 (без отделки)</v>
+        <v>0 (стяжка)</v>
       </c>
       <c r="AG9" s="1" t="str">
         <v>Самая низкая цена в Ставрополе</v>
@@ -3487,9 +3502,15 @@
       <c r="D30" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E30" s="1" t="str">
+        <v>СЗ Ставропольская Строительная Компания</v>
+      </c>
       <c r="L30" s="1" t="str">
         <v>Пятигорск</v>
       </c>
+      <c r="M30" s="1" t="str">
+        <v>ул. Ессентукская</v>
+      </c>
       <c r="N30" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -3513,6 +3534,9 @@
       </c>
       <c r="AD30" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF30" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG30" s="1" t="str">
         <v>Панорамные окна</v>
@@ -3555,9 +3579,15 @@
       <c r="D31" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E31" s="1" t="str">
+        <v>Развитие Курортов</v>
+      </c>
       <c r="L31" s="1" t="str">
         <v>Пятигорск</v>
       </c>
+      <c r="M31" s="1" t="str">
+        <v>ул. Ермолова, 28/1</v>
+      </c>
       <c r="N31" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -3565,7 +3595,13 @@
         <v>Строится</v>
       </c>
       <c r="P31" s="1" t="str">
-        <v>3 кв.2027-2 кв.2028</v>
+        <v>1 кв.2028-2 кв.2029</v>
+      </c>
+      <c r="Q31" s="1" t="str">
+        <v>5</v>
+      </c>
+      <c r="R31" s="1" t="str">
+        <v>10</v>
       </c>
       <c r="S31" s="1" t="str">
         <v>217</v>
@@ -3587,6 +3623,9 @@
       </c>
       <c r="AD31" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF31" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG31" s="1" t="str">
         <v>Низкая цена от 3,5 млн</v>
@@ -3629,23 +3668,35 @@
       <c r="D32" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E32" s="1" t="str">
+        <v>СЗ СПЕЦСТРОЙМОНТАЖ</v>
+      </c>
       <c r="L32" s="1" t="str">
         <v>Пятигорск</v>
       </c>
+      <c r="M32" s="1" t="str">
+        <v>пр. Калинина / ул. Первомайская</v>
+      </c>
       <c r="N32" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O32" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P32" s="1" t="str">
+        <v>2029</v>
+      </c>
       <c r="Q32" s="1" t="str">
         <v>1</v>
       </c>
       <c r="R32" s="1" t="str">
-        <v>16</v>
+        <v>4-18</v>
       </c>
       <c r="AD32" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF32" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG32" s="1" t="str">
         <v>16 этажей</v>
@@ -3688,6 +3739,9 @@
       <c r="D33" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E33" s="1" t="str">
+        <v>СЗ Курортный</v>
+      </c>
       <c r="L33" s="1" t="str">
         <v>Пятигорск</v>
       </c>
@@ -3697,6 +3751,9 @@
       <c r="O33" s="1" t="str">
         <v>Строится/сдан</v>
       </c>
+      <c r="P33" s="1" t="str">
+        <v>2026-2027</v>
+      </c>
       <c r="U33" s="1" t="str">
         <v>36,2</v>
       </c>
@@ -3714,6 +3771,9 @@
       </c>
       <c r="AD33" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF33" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG33" s="1" t="str">
         <v>Рядом с озёрами</v>
@@ -3753,6 +3813,9 @@
       <c r="D34" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E34" s="1" t="str">
+        <v>Аксиома-СЗ</v>
+      </c>
       <c r="L34" s="1" t="str">
         <v>Пятигорск</v>
       </c>
@@ -3762,6 +3825,12 @@
       <c r="O34" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P34" s="1" t="str">
+        <v>III кв.2026</v>
+      </c>
+      <c r="R34" s="1" t="str">
+        <v>13</v>
+      </c>
       <c r="U34" s="1" t="str">
         <v>42,4</v>
       </c>
@@ -3779,6 +3848,9 @@
       </c>
       <c r="AD34" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF34" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG34" s="1" t="str">
         <v>Современный минимализм</v>
@@ -3821,6 +3893,9 @@
       <c r="D35" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E35" s="1" t="str">
+        <v>СК Олимп</v>
+      </c>
       <c r="L35" s="1" t="str">
         <v>Ессентуки</v>
       </c>
@@ -3830,8 +3905,11 @@
       <c r="O35" s="1" t="str">
         <v>Строится/сдан</v>
       </c>
+      <c r="P35" s="1" t="str">
+        <v>сдан/строится</v>
+      </c>
       <c r="Q35" s="1" t="str">
-        <v>14 (10 сданы)</v>
+        <v>14</v>
       </c>
       <c r="R35" s="1" t="str">
         <v>разная</v>
@@ -3853,6 +3931,9 @@
       </c>
       <c r="AD35" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF35" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG35" s="1" t="str">
         <v>14 корпусов — город в городе</v>
@@ -3895,6 +3976,9 @@
       <c r="D36" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E36" s="1" t="str">
+        <v>Наследие</v>
+      </c>
       <c r="L36" s="1" t="str">
         <v>Ессентуки</v>
       </c>
@@ -3904,6 +3988,9 @@
       <c r="O36" s="1" t="str">
         <v>Строится/сдан</v>
       </c>
+      <c r="P36" s="1" t="str">
+        <v>2025-2026</v>
+      </c>
       <c r="U36" s="1" t="str">
         <v>45,7</v>
       </c>
@@ -3921,6 +4008,9 @@
       </c>
       <c r="AD36" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF36" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG36" s="1" t="str">
         <v>Набережная реки</v>
@@ -3963,15 +4053,33 @@
       <c r="D37" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E37" s="1" t="str">
+        <v>СЗ Николаевский</v>
+      </c>
       <c r="L37" s="1" t="str">
         <v>Ессентуки</v>
       </c>
+      <c r="M37" s="1" t="str">
+        <v>ул. Благодатная</v>
+      </c>
       <c r="N37" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O37" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P37" s="1" t="str">
+        <v>2028</v>
+      </c>
+      <c r="Q37" s="1" t="str">
+        <v>7</v>
+      </c>
+      <c r="R37" s="1" t="str">
+        <v>9</v>
+      </c>
+      <c r="S37" s="1" t="str">
+        <v>820</v>
+      </c>
       <c r="U37" s="1" t="str">
         <v>37,1</v>
       </c>
@@ -3989,6 +4097,9 @@
       </c>
       <c r="AD37" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF37" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG37" s="1" t="str">
         <v>Цены от 4,8 млн</v>
@@ -4031,9 +4142,15 @@
       <c r="D38" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E38" s="1" t="str">
+        <v>КВС (Клуб Высотного Строительства)</v>
+      </c>
       <c r="L38" s="1" t="str">
         <v>Ессентуки</v>
       </c>
+      <c r="M38" s="1" t="str">
+        <v>ул. Буачидзе</v>
+      </c>
       <c r="N38" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -4063,6 +4180,9 @@
       </c>
       <c r="AD38" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF38" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG38" s="1" t="str">
         <v>ул. Буачидзе — центр Ессентуков</v>
@@ -4105,17 +4225,29 @@
       <c r="D39" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E39" s="1" t="str">
+        <v>застройщик не указан</v>
+      </c>
       <c r="L39" s="1" t="str">
         <v>Ессентуки</v>
       </c>
+      <c r="M39" s="1" t="str">
+        <v>ул. Галерейная</v>
+      </c>
       <c r="N39" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O39" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P39" s="1" t="str">
+        <v>2026-2027</v>
+      </c>
       <c r="AD39" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF39" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG39" s="1" t="str">
         <v>Спортивные площадки</v>
@@ -4155,15 +4287,27 @@
       <c r="D40" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E40" s="1" t="str">
+        <v>СЗ Печорин</v>
+      </c>
       <c r="L40" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M40" s="1" t="str">
+        <v>Берёзовское ущелье</v>
+      </c>
       <c r="N40" s="1" t="str">
         <v>Клубный</v>
       </c>
       <c r="O40" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="Q40" s="1" t="str">
+        <v>5</v>
+      </c>
+      <c r="R40" s="1" t="str">
+        <v>6</v>
+      </c>
       <c r="U40" s="1" t="str">
         <v>86</v>
       </c>
@@ -4181,6 +4325,9 @@
       </c>
       <c r="AD40" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF40" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG40" s="1" t="str">
         <v>Закрытый клубный квартал</v>
@@ -4223,9 +4370,15 @@
       <c r="D41" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E41" s="1" t="str">
+        <v>СЗ Реликт</v>
+      </c>
       <c r="L41" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M41" s="1" t="str">
+        <v>Кисловодск</v>
+      </c>
       <c r="N41" s="1" t="str">
         <v>Премиум</v>
       </c>
@@ -4249,6 +4402,9 @@
       </c>
       <c r="AD41" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF41" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG41" s="1" t="str">
         <v>Премиум с отделкой под ключ</v>
@@ -4291,9 +4447,15 @@
       <c r="D42" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E42" s="1" t="str">
+        <v>ИП Тамаев А.А.</v>
+      </c>
       <c r="L42" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M42" s="1" t="str">
+        <v>ул. Московская</v>
+      </c>
       <c r="N42" s="1" t="str">
         <v>Элитный</v>
       </c>
@@ -4308,6 +4470,9 @@
       </c>
       <c r="AD42" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF42" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG42" s="1" t="str">
         <v>Центр Кисловодска</v>
@@ -4350,17 +4515,38 @@
       <c r="D43" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E43" s="1" t="str">
+        <v>СЗ Виноград</v>
+      </c>
       <c r="L43" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M43" s="1" t="str">
+        <v>Кисловодск</v>
+      </c>
       <c r="N43" s="1" t="str">
-        <v>Премиум</v>
+        <v>Бизнес</v>
       </c>
       <c r="O43" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P43" s="1" t="str">
+        <v>IV кв.2026</v>
+      </c>
+      <c r="R43" s="1" t="str">
+        <v>9</v>
+      </c>
+      <c r="U43" s="1" t="str">
+        <v>56</v>
+      </c>
+      <c r="W43" s="1" t="str">
+        <v>1к/2к/3к</v>
+      </c>
       <c r="AD43" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF43" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG43" s="1" t="str">
         <v>Курортный парк рядом</v>
@@ -4403,6 +4589,9 @@
       <c r="D44" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E44" s="1" t="str">
+        <v>СЗ Моя Легенда</v>
+      </c>
       <c r="L44" s="1" t="str">
         <v>Кисловодск</v>
       </c>
@@ -4432,6 +4621,9 @@
       </c>
       <c r="AD44" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF44" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG44" s="1" t="str">
         <v>Кладовые помещения</v>
@@ -4474,15 +4666,30 @@
       <c r="D45" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E45" s="1" t="str">
+        <v>ЮгСтройИнвест (ЮСИ)</v>
+      </c>
       <c r="L45" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M45" s="1" t="str">
+        <v>пос. Аликоновка</v>
+      </c>
       <c r="N45" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O45" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P45" s="1" t="str">
+        <v>2027-2028</v>
+      </c>
+      <c r="Q45" s="1" t="str">
+        <v>4</v>
+      </c>
+      <c r="R45" s="1" t="str">
+        <v>4-14</v>
+      </c>
       <c r="U45" s="1" t="str">
         <v>35</v>
       </c>
@@ -4500,6 +4707,9 @@
       </c>
       <c r="AD45" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF45" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG45" s="1" t="str">
         <v>Расположение у озера</v>
@@ -4542,9 +4752,15 @@
       <c r="D46" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E46" s="1" t="str">
+        <v>ССК</v>
+      </c>
       <c r="L46" s="1" t="str">
         <v>Железноводск</v>
       </c>
+      <c r="M46" s="1" t="str">
+        <v>Железноводский р-н</v>
+      </c>
       <c r="N46" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -4554,6 +4770,12 @@
       <c r="P46" s="1" t="str">
         <v>2 кв.2029</v>
       </c>
+      <c r="Q46" s="1" t="str">
+        <v>22 квартала</v>
+      </c>
+      <c r="R46" s="1" t="str">
+        <v>9-14</v>
+      </c>
       <c r="S46" s="1" t="str">
         <v>637</v>
       </c>
@@ -4574,6 +4796,9 @@
       </c>
       <c r="AD46" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF46" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG46" s="1" t="str">
         <v>150 га у подножия гор</v>
@@ -4616,6 +4841,9 @@
       <c r="D47" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E47" s="1" t="str">
+        <v>СЗ Живописный</v>
+      </c>
       <c r="L47" s="1" t="str">
         <v>Железноводск</v>
       </c>
@@ -4648,6 +4876,9 @@
       </c>
       <c r="AD47" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF47" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG47" s="1" t="str">
         <v>Скоро — 3 кв.2026</v>
@@ -4690,17 +4921,29 @@
       <c r="D48" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E48" s="1" t="str">
+        <v>AVA Group</v>
+      </c>
       <c r="L48" s="1" t="str">
         <v>п. Джуца (Предгорный окр.)</v>
       </c>
+      <c r="M48" s="1" t="str">
+        <v>п. Джуца, Ореховая ул.</v>
+      </c>
       <c r="N48" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O48" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="P48" s="1" t="str">
+        <v>2028-2029</v>
+      </c>
+      <c r="Q48" s="1" t="str">
+        <v>7</v>
+      </c>
       <c r="R48" s="1" t="str">
-        <v>15</v>
+        <v>12-15</v>
       </c>
       <c r="U48" s="1" t="str">
         <v>22,3</v>
@@ -4719,6 +4962,9 @@
       </c>
       <c r="AD48" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF48" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG48" s="1" t="str">
         <v>15-этажные монолитные дома</v>
@@ -4761,15 +5007,24 @@
       <c r="D49" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E49" s="1" t="str">
+        <v>EFFECT Development</v>
+      </c>
       <c r="L49" s="1" t="str">
         <v>ст. Ессентукская</v>
       </c>
+      <c r="M49" s="1" t="str">
+        <v>ст. Ессентукская</v>
+      </c>
       <c r="N49" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O49" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="R49" s="1" t="str">
+        <v>4</v>
+      </c>
       <c r="U49" s="1" t="str">
         <v>37,5</v>
       </c>
@@ -4784,6 +5039,9 @@
       </c>
       <c r="AD49" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF49" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG49" s="1" t="str">
         <v>Премиум в сердце КМВ</v>
@@ -4826,9 +5084,15 @@
       <c r="D50" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E50" s="1" t="str">
+        <v>СЗ Резиденция</v>
+      </c>
       <c r="L50" s="1" t="str">
         <v>Лермонтов</v>
       </c>
+      <c r="M50" s="1" t="str">
+        <v>Лермонтов</v>
+      </c>
       <c r="N50" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -4852,6 +5116,9 @@
       </c>
       <c r="AD50" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF50" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG50" s="1" t="str">
         <v>Беспроцентная рассрочка</v>
@@ -4894,9 +5161,15 @@
       <c r="D51" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E51" s="1" t="str">
+        <v>СЗ Радонежская</v>
+      </c>
       <c r="L51" s="1" t="str">
         <v>Лермонтов</v>
       </c>
+      <c r="M51" s="1" t="str">
+        <v>ул. Радонежская, Лермонтов</v>
+      </c>
       <c r="N51" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -4920,6 +5193,9 @@
       </c>
       <c r="AD51" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF51" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG51" s="1" t="str">
         <v>Цена от 4,7 млн</v>
@@ -4959,15 +5235,24 @@
       <c r="D52" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E52" s="1" t="str">
+        <v>СЗ Кристалл-Георгиевск</v>
+      </c>
       <c r="L52" s="1" t="str">
         <v>Георгиевск</v>
       </c>
+      <c r="M52" s="1" t="str">
+        <v>Георгиевск</v>
+      </c>
       <c r="N52" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O52" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="Q52" s="1" t="str">
+        <v>1</v>
+      </c>
       <c r="R52" s="1" t="str">
         <v>16</v>
       </c>
@@ -4991,6 +5276,9 @@
       </c>
       <c r="AD52" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF52" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG52" s="1" t="str">
         <v>Самая низкая цена — от 3 млн</v>
@@ -5033,18 +5321,30 @@
       <c r="D53" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E53" s="1" t="str">
+        <v>СЗ Олимп</v>
+      </c>
       <c r="L53" s="1" t="str">
         <v>Георгиевск</v>
       </c>
+      <c r="M53" s="1" t="str">
+        <v>ул. Филатова, Георгиевск</v>
+      </c>
       <c r="N53" s="1" t="str">
         <v>Комфорт</v>
       </c>
       <c r="O53" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="X53" s="1" t="str">
+        <v>3 970 000</v>
+      </c>
       <c r="AD53" s="1" t="str">
         <v>май 2026</v>
       </c>
+      <c r="AF53" s="1" t="str">
+        <v>2 000-5 000</v>
+      </c>
       <c r="AG53" s="1" t="str">
         <v>ул. Филатова</v>
       </c>
@@ -5067,7 +5367,7 @@
         <v>7%</v>
       </c>
       <c r="AN53" s="1" t="str">
-        <v>нет</v>
+        <v>беспроцентная</v>
       </c>
       <c r="AO53" s="1" t="str">
         <v>6%</v>
@@ -5086,9 +5386,15 @@
       <c r="D54" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E54" s="1" t="str">
+        <v>СЗ Садовое Кольцо</v>
+      </c>
       <c r="L54" s="1" t="str">
         <v>ст. Ессентукская</v>
       </c>
+      <c r="M54" s="1" t="str">
+        <v>ст. Ессентукская, ул. Садовое Кольцо</v>
+      </c>
       <c r="N54" s="1" t="str">
         <v>Комфорт</v>
       </c>
@@ -5112,6 +5418,9 @@
       </c>
       <c r="AD54" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF54" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG54" s="1" t="str">
         <v>Станица Ессентукская</v>
@@ -5151,17 +5460,32 @@
       <c r="D55" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E55" s="1" t="str">
+        <v>КВС (Клуб Высотного Строительства)</v>
+      </c>
       <c r="L55" s="1" t="str">
         <v>Ессентуки</v>
       </c>
+      <c r="M55" s="1" t="str">
+        <v>ул. Буачидзе, Ессентуки</v>
+      </c>
       <c r="N55" s="1" t="str">
         <v>Бизнес</v>
       </c>
       <c r="O55" s="1" t="str">
         <v>Строится/сдан</v>
       </c>
+      <c r="X55" s="1" t="str">
+        <v>7 000 000</v>
+      </c>
+      <c r="Y55" s="1" t="str">
+        <v>12 000 000</v>
+      </c>
       <c r="AD55" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF55" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG55" s="1" t="str">
         <v>Бизнес-класс, центр Ессентуков</v>
@@ -5207,6 +5531,9 @@
       <c r="L56" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M56" s="1" t="str">
+        <v>ул. Клары Цеткин, Кисловодск</v>
+      </c>
       <c r="N56" s="1" t="str">
         <v>Элитный</v>
       </c>
@@ -5218,6 +5545,9 @@
       </c>
       <c r="AD56" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF56" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG56" s="1" t="str">
         <v>Элитный 9 этажей</v>
@@ -5263,6 +5593,9 @@
       <c r="L57" s="1" t="str">
         <v>Кисловодск</v>
       </c>
+      <c r="M57" s="1" t="str">
+        <v>Кисловодск</v>
+      </c>
       <c r="N57" s="1" t="str">
         <v>Апартаменты</v>
       </c>
@@ -5289,6 +5622,9 @@
       </c>
       <c r="AD57" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF57" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG57" s="1" t="str">
         <v>Апарт-отель — инвестиции</v>
@@ -5331,17 +5667,29 @@
       <c r="D58" s="1" t="str">
         <v>Активные продажи</v>
       </c>
+      <c r="E58" s="1" t="str">
+        <v>СЗ Филатова</v>
+      </c>
       <c r="L58" s="1" t="str">
         <v>Георгиевск</v>
       </c>
+      <c r="M58" s="1" t="str">
+        <v>ул. Филатова, Георгиевск</v>
+      </c>
       <c r="N58" s="1" t="str">
         <v>Эконом</v>
       </c>
       <c r="O58" s="1" t="str">
         <v>Строится</v>
       </c>
+      <c r="X58" s="1" t="str">
+        <v>3 500 000</v>
+      </c>
       <c r="AD58" s="1" t="str">
         <v>май 2026</v>
+      </c>
+      <c r="AF58" s="1" t="str">
+        <v>2 000-5 000</v>
       </c>
       <c r="AG58" s="1" t="str">
         <v>Самая низкая цена — эконом</v>

</xml_diff>